<commit_message>
Fix ISEQL operators to ICSC 2016 and regenerate evaluation data
Align all 8 ISEQL operators to the ICSC 2016 original paper semantics,
fix End Following to use epsilon (not delta per CIKM 2017 error),
correct fight sound query to SoundClass='impact' only, fix no-reID
AnalysisID bug, rewrite ISEQL helpers with r/s parameter naming.

Regenerate all evaluation xlsx via standalone scripts and notebook
re-runs: visual A (offline), audio B (window/hop ablation, 16 combos),
multimodal C (64 combos across VLM×audio×window/hop). Add frontend
configurable audio window/hop and VLM model defaults per provider.
Remove dead deltas from frontend and align evaluation_scenes.md ISEQL
patterns with current query semantics.
</commit_message>
<xml_diff>
--- a/data/analysis_gemini_2_5_flash/summary.xlsx
+++ b/data/analysis_gemini_2_5_flash/summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>provider</t>
   </si>
@@ -35,12 +35,6 @@
   </si>
   <si>
     <t>FN</t>
-  </si>
-  <si>
-    <t>support</t>
-  </si>
-  <si>
-    <t>VPI</t>
   </si>
   <si>
     <t>gemini_2_5_flash</t>
@@ -50,8 +44,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -67,7 +69,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -75,12 +77,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -375,65 +395,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
       <c r="B2">
-        <v>0.826</v>
+        <v>0.842</v>
       </c>
       <c r="C2">
-        <v>0.633</v>
+        <v>0.533</v>
       </c>
       <c r="D2">
-        <v>0.717</v>
+        <v>0.653</v>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>11</v>
-      </c>
-      <c r="H2">
-        <v>30</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restructure evaluation tables, slides, and documentation
Standardize summary.xlsx schemas: visual (visual/reid/precision/recall/
f1/TP/FP/FN/support/VPI), multimodal (visual/reid/audio/window/hop/
precision/recall/f1/TP/FP/FN/support/VPI/SPI), audio (audio/window/hop/
precision/recall/f1/TP/FP/FN/support/SPI). Remove provider column.

Redesign slides: expand RQ3 to full per-pair metrics table, add complete
64-combo appendix (4 frames A-1/A-4), redesign RQ1/RQ2/RQ3 slide layouts.

Update thesis/slides/README table headers: Provider→Model,
VLM+Audio→VLM+Audio Model, Win(s)→Window(s), split TP/FP/FN into
separate columns. Replace em-dashes with colons/commas in docs and
scene descriptions. Bold best rows in evaluation tables.
</commit_message>
<xml_diff>
--- a/data/analysis_gemini_2_5_flash/summary.xlsx
+++ b/data/analysis_gemini_2_5_flash/summary.xlsx
@@ -14,9 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>provider</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>visual</t>
+  </si>
+  <si>
+    <t>reid</t>
   </si>
   <si>
     <t>precision</t>
@@ -35,6 +38,12 @@
   </si>
   <si>
     <t>FN</t>
+  </si>
+  <si>
+    <t>support</t>
+  </si>
+  <si>
+    <t>VPI</t>
   </si>
   <si>
     <t>gemini_2_5_flash</t>
@@ -44,16 +53,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -69,7 +70,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -77,30 +78,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -395,53 +378,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>0.842</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>0.533</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>0.653</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>16</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>3</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>14</v>
+      </c>
+      <c r="I2">
+        <v>30</v>
+      </c>
+      <c r="J2">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Convert thesis figures to B&W and change loitering threshold to 120
Convert 3 thesis figures to formal black-and-white style: fill=white,
draw=black, sharp corners, simplified titles. Remove unused figure
files. Reduce pipeline figure width from 0.55 to 0.40 textwidth.

Change delta_visual_loitering from 150 to 120 frames (5.0 s at 24 fps)
in backend defaults, frontend fallback, eval scripts, and all 16
notebooks. Regenerate visual (A) and multimodal (C) evaluation data
offline. Update all thesis tables (5.1/5.3/5.4/5.5), slides appendix,
README, ISEQL query docs, evaluation_scenes.md, and research proposal.
Restore pipeline figures to 0.40textwidth. Replace \S with Section~\ref.
</commit_message>
<xml_diff>
--- a/data/analysis_gemini_2_5_flash/summary.xlsx
+++ b/data/analysis_gemini_2_5_flash/summary.xlsx
@@ -53,8 +53,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -70,7 +78,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -78,12 +86,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -382,34 +408,34 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -421,22 +447,22 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.842</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="D2">
-        <v>0.533</v>
+        <v>0.6</v>
       </c>
       <c r="E2">
-        <v>0.653</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I2">
         <v>30</v>

</xml_diff>